<commit_message>
Actualizacion en Apartado de Matematica Discreta
Se añadio el nuevas funcionalidades
</commit_message>
<xml_diff>
--- a/Proyecto_Final_Unificado - UMG/Matematica Discreta/datos_mate_discreta.xlsx
+++ b/Proyecto_Final_Unificado - UMG/Matematica Discreta/datos_mate_discreta.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -598,6 +598,25 @@
       </c>
       <c r="E9" t="n">
         <v>10</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>45955.06937489584</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>combinaciones</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -611,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -888,6 +907,706 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>A ⊆ B  →  False</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>45955.06659457176</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>a ∩ b</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>A,B,C,3,4,5</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>{A, B, C}</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>45955.06665121527</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>b ∪ a</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>A,B,C,3,4,5</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>{3, 4, 5, A, B, C, D, E, F}</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>45955.06685633102</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>b △ a</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>A,B,C,3,4,5</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>{3, 4, 5, D, E, F}</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>45955.06899105324</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>b − a</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G,H,I,1,2,3,4</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>A,F,D,2,4,5</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>{5}</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>45955.06903230324</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>a ∪ b</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G,H,I,1,2,3,4</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>A,F,D,2,4,5</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>{1, 2, 3, 4, 5, A, B, C, D, E, F, G, H, I}</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>45955.06906487269</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>a ∩ b</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G,H,I,1,2,3,4</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>A,F,D,2,4,5</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>{2, 4, A, D, F}</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>45955.06909590278</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>subconjunto</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G,H,I,1,2,3,4</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>A,F,D,2,4,5</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>B ⊆ A  →  False</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>45955.06912611111</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>subconjunto</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G,H,I,1,2,3,4</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>A,F,D,2,4,5</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>A ⊆ B  →  False</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
+        <v>45955.06922752315</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>subconjunto</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G,H,I,1,2,3,4</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>A,B,C</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>B ⊆ A  →  True</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="n">
+        <v>45955.0694393287</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>a ∪ b</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G,H,I,1,2,3,4</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>A,B,C</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>{1, 2, 3, 4, A, B, C, D, E, F, G, H, I}</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>45955.06943989584</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>a ∩ b</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G,H,I,1,2,3,4</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>A,B,C</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>{A, B, C}</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>45955.06944032407</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>a − b</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G,H,I,1,2,3,4</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>A,B,C</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>{1, 2, 3, 4, D, E, F, G, H, I}</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>45955.06944075231</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>a △ b</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G,H,I,1,2,3,4</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>A,B,C</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>{1, 2, 3, 4, D, E, F, G, H, I}</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>45955.06944118055</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>subconjunto</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>A,B,C,D,E,F,G,H,I,1,2,3,4</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>A,B,C</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>A ⊆ B  →  False</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>45955.07087193287</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>a ∪ b</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>a,b,c,d,e,1,2,3</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>{1, 2, 3, a, b, c, d, e}</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>45955.07087239583</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>a ∩ b</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>a,b,c,d,e,1,2,3</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>{1, 2, 3}</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>45955.07087284722</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>a − b</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>a,b,c,d,e,1,2,3</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>{a, b, c, d, e}</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="n">
+        <v>45955.07087328703</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>b − a</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>a,b,c,d,e,1,2,3</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="n">
+        <v>45955.07087373843</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>a △ b</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>a,b,c,d,e,1,2,3</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>{a, b, c, d, e}</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="n">
+        <v>45955.07087418981</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>subconjunto</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>a,b,c,d,e,1,2,3</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>A ⊆ B  →  False</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="n">
+        <v>45955.07087464121</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>subconjunto</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>a,b,c,d,e,1,2,3</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>B ⊆ A  →  True</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="n">
+        <v>45955.07093056713</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>a ∪ b</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>a,b,c,d,e,1,2,3</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>{1, 2, 3, a, b, c, d, e}</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>45955.07095231482</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>a ∩ b</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>a,b,c,d,e,1,2,3</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>{1, 2, 3}</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="n">
+        <v>45955.0709743287</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>a − b</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>a,b,c,d,e,1,2,3</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>{a, b, c, d, e}</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>45955.07099559028</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>b − a</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>a,b,c,d,e,1,2,3</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n">
+        <v>45955.0710328588</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>a △ b</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>a,b,c,d,e,1,2,3</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>{a, b, c, d, e}</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="n">
+        <v>45955.07113427083</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>subconjunto</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>a,b,c,d,e,1,2,3</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>A ⊆ B  →  False</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n">
+        <v>45955.07116565719</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>subconjunto</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>a,b,c,d,e,1,2,3</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>B ⊆ A  →  True</t>
         </is>
       </c>
     </row>
@@ -1029,7 +1748,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>45955.01905740133</v>
+        <v>45955.01905739583</v>
       </c>
       <c r="B7" t="n">
         <v>12</v>

</xml_diff>